<commit_message>
Add correct score odds and complete DNB for all matches
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backtest_v3.xlsx
+++ b/backtest_v3.xlsx
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.50</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -7219,7 +7219,7 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="E127" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F127" s="3" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.88</t>
         </is>
       </c>
       <c r="F131" s="3" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F137" s="3" t="inlineStr">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.50</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F139" s="3" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F142" s="5" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F143" s="3" t="inlineStr">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
@@ -9416,7 +9416,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.50</t>
         </is>
       </c>
       <c r="F170" s="5" t="inlineStr">
@@ -9453,7 +9453,7 @@
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F171" s="3" t="inlineStr">
@@ -9490,7 +9490,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F172" s="5" t="inlineStr">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F173" s="3" t="inlineStr">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F174" s="5" t="inlineStr">
@@ -9601,7 +9601,7 @@
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F175" s="3" t="inlineStr">
@@ -9638,7 +9638,7 @@
       </c>
       <c r="E176" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F176" s="5" t="inlineStr">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F179" s="3" t="inlineStr">
@@ -10718,7 +10718,7 @@
       </c>
       <c r="E207" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F207" s="3" t="inlineStr">
@@ -10792,7 +10792,7 @@
       </c>
       <c r="E209" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F209" s="3" t="inlineStr">
@@ -10829,7 +10829,7 @@
       </c>
       <c r="E210" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F210" s="5" t="inlineStr">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="E211" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F211" s="3" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="E212" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F212" s="5" t="inlineStr">
@@ -10940,7 +10940,7 @@
       </c>
       <c r="E213" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F213" s="3" t="inlineStr">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="E214" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F214" s="5" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="E215" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F215" s="3" t="inlineStr">
@@ -11909,7 +11909,7 @@
       </c>
       <c r="E241" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.50</t>
         </is>
       </c>
       <c r="F241" s="3" t="inlineStr">
@@ -11983,7 +11983,7 @@
       </c>
       <c r="E243" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F243" s="3" t="inlineStr">
@@ -12020,7 +12020,7 @@
       </c>
       <c r="E244" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F244" s="5" t="inlineStr">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="E245" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F245" s="3" t="inlineStr">
@@ -12094,7 +12094,7 @@
       </c>
       <c r="E246" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F246" s="5" t="inlineStr">
@@ -12131,7 +12131,7 @@
       </c>
       <c r="E247" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F247" s="3" t="inlineStr">
@@ -12168,7 +12168,7 @@
       </c>
       <c r="E248" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F248" s="5" t="inlineStr">
@@ -12205,7 +12205,7 @@
       </c>
       <c r="E249" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F249" s="3" t="inlineStr">
@@ -13174,7 +13174,7 @@
       </c>
       <c r="E277" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F277" s="3" t="inlineStr">
@@ -13211,7 +13211,7 @@
       </c>
       <c r="E278" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F278" s="5" t="inlineStr">
@@ -13248,7 +13248,7 @@
       </c>
       <c r="E279" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F279" s="3" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="E280" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.50</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
@@ -13322,7 +13322,7 @@
       </c>
       <c r="E281" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F281" s="3" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="E282" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="E283" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="F283" s="3" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="E284" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
@@ -14291,7 +14291,7 @@
       </c>
       <c r="E309" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F309" s="3" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="E310" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="F310" s="5" t="inlineStr">
@@ -14365,7 +14365,7 @@
       </c>
       <c r="E311" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>34.00</t>
         </is>
       </c>
       <c r="F311" s="3" t="inlineStr">
@@ -14402,7 +14402,7 @@
       </c>
       <c r="E312" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F312" s="5" t="inlineStr">
@@ -14439,7 +14439,7 @@
       </c>
       <c r="E313" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F313" s="3" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="E316" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F316" s="5" t="inlineStr">
@@ -14794,37 +14794,37 @@
       </c>
     </row>
     <row r="325" ht="15" customHeight="1">
-      <c r="A325" s="22" t="inlineStr">
+      <c r="A325" s="17" t="inlineStr">
         <is>
           <t>Netherlands vs Japan</t>
         </is>
       </c>
-      <c r="B325" s="22" t="inlineStr">
-        <is>
-          <t>Double Chance X2 *** ACCUMULATOR</t>
-        </is>
-      </c>
-      <c r="C325" s="23" t="inlineStr">
+      <c r="B325" s="17" t="inlineStr">
+        <is>
+          <t>Double Chance X2</t>
+        </is>
+      </c>
+      <c r="C325" s="3" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="D325" s="23" t="inlineStr">
+      <c r="D325" s="15" t="inlineStr">
         <is>
           <t>74.1%</t>
         </is>
       </c>
-      <c r="E325" s="23" t="inlineStr">
+      <c r="E325" s="3" t="inlineStr">
         <is>
           <t>1.80</t>
         </is>
       </c>
-      <c r="F325" s="23" t="inlineStr">
+      <c r="F325" s="3" t="inlineStr">
         <is>
           <t>dc</t>
         </is>
       </c>
-      <c r="G325" s="23" t="inlineStr">
+      <c r="G325" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -15164,37 +15164,37 @@
       </c>
     </row>
     <row r="335" ht="15" customHeight="1">
-      <c r="A335" s="17" t="inlineStr">
+      <c r="A335" s="22" t="inlineStr">
         <is>
           <t>Netherlands vs Japan</t>
         </is>
       </c>
-      <c r="B335" s="17" t="inlineStr">
-        <is>
-          <t>Draw No Bet Japan</t>
-        </is>
-      </c>
-      <c r="C335" s="3" t="inlineStr">
+      <c r="B335" s="22" t="inlineStr">
+        <is>
+          <t>Draw No Bet Japan *** ACCUMULATOR</t>
+        </is>
+      </c>
+      <c r="C335" s="23" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="D335" s="11" t="inlineStr">
+      <c r="D335" s="23" t="inlineStr">
         <is>
           <t>57.3%</t>
         </is>
       </c>
-      <c r="E335" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F335" s="3" t="inlineStr">
+      <c r="E335" s="23" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="F335" s="23" t="inlineStr">
         <is>
           <t>dnb</t>
         </is>
       </c>
-      <c r="G335" s="3" t="inlineStr">
+      <c r="G335" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -15408,7 +15408,7 @@
       </c>
       <c r="E341" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F341" s="3" t="inlineStr">
@@ -15704,7 +15704,7 @@
       </c>
       <c r="E349" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F349" s="3" t="inlineStr">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="E350" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F350" s="5" t="inlineStr">
@@ -15778,7 +15778,7 @@
       </c>
       <c r="E351" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F351" s="3" t="inlineStr">
@@ -15815,7 +15815,7 @@
       </c>
       <c r="E352" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F352" s="5" t="inlineStr">
@@ -15852,7 +15852,7 @@
       </c>
       <c r="E353" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F353" s="3" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="E354" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F354" s="5" t="inlineStr">
@@ -15926,7 +15926,7 @@
       </c>
       <c r="E355" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F355" s="3" t="inlineStr">
@@ -15963,7 +15963,7 @@
       </c>
       <c r="E356" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F356" s="5" t="inlineStr">
@@ -16562,7 +16562,7 @@
       </c>
       <c r="E374" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="F374" s="5" t="inlineStr">
@@ -16747,7 +16747,7 @@
       </c>
       <c r="E379" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F379" s="3" t="inlineStr">
@@ -16932,7 +16932,7 @@
       </c>
       <c r="E384" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F384" s="5" t="inlineStr">
@@ -16969,7 +16969,7 @@
       </c>
       <c r="E385" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F385" s="3" t="inlineStr">
@@ -17006,7 +17006,7 @@
       </c>
       <c r="E386" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F386" s="5" t="inlineStr">
@@ -17043,7 +17043,7 @@
       </c>
       <c r="E387" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.50</t>
         </is>
       </c>
       <c r="F387" s="3" t="inlineStr">
@@ -17080,7 +17080,7 @@
       </c>
       <c r="E388" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F388" s="5" t="inlineStr">
@@ -17117,7 +17117,7 @@
       </c>
       <c r="E389" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F389" s="3" t="inlineStr">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="E390" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="F390" s="5" t="inlineStr">
@@ -17191,7 +17191,7 @@
       </c>
       <c r="E391" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F391" s="3" t="inlineStr">
@@ -17420,7 +17420,7 @@
       </c>
       <c r="E399" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="F399" s="3" t="inlineStr">
@@ -18049,7 +18049,7 @@
       </c>
       <c r="E416" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="F416" s="5" t="inlineStr">
@@ -18160,7 +18160,7 @@
       </c>
       <c r="E419" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F419" s="3" t="inlineStr">
@@ -18197,7 +18197,7 @@
       </c>
       <c r="E420" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F420" s="5" t="inlineStr">
@@ -18234,7 +18234,7 @@
       </c>
       <c r="E421" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F421" s="3" t="inlineStr">
@@ -18271,7 +18271,7 @@
       </c>
       <c r="E422" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F422" s="5" t="inlineStr">
@@ -18308,7 +18308,7 @@
       </c>
       <c r="E423" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.50</t>
         </is>
       </c>
       <c r="F423" s="3" t="inlineStr">
@@ -18345,7 +18345,7 @@
       </c>
       <c r="E424" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16.00</t>
         </is>
       </c>
       <c r="F424" s="5" t="inlineStr">
@@ -18382,7 +18382,7 @@
       </c>
       <c r="E425" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F425" s="3" t="inlineStr">
@@ -18419,7 +18419,7 @@
       </c>
       <c r="E426" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>22.00</t>
         </is>
       </c>
       <c r="F426" s="5" t="inlineStr">
@@ -18500,7 +18500,7 @@
       </c>
       <c r="E430" s="23" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="F430" s="23" t="inlineStr">
@@ -19351,7 +19351,7 @@
       </c>
       <c r="E453" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F453" s="3" t="inlineStr">
@@ -19388,7 +19388,7 @@
       </c>
       <c r="E454" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F454" s="5" t="inlineStr">
@@ -19425,7 +19425,7 @@
       </c>
       <c r="E455" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="F455" s="3" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="E456" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="F456" s="5" t="inlineStr">
@@ -19499,7 +19499,7 @@
       </c>
       <c r="E457" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F457" s="3" t="inlineStr">
@@ -19536,7 +19536,7 @@
       </c>
       <c r="E458" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>23.00</t>
         </is>
       </c>
       <c r="F458" s="5" t="inlineStr">
@@ -19573,7 +19573,7 @@
       </c>
       <c r="E459" s="3" t="inlineStr">
         <is>
-          <t>12.00</t>
+          <t>18.00</t>
         </is>
       </c>
       <c r="F459" s="3" t="inlineStr">
@@ -19610,7 +19610,7 @@
       </c>
       <c r="E460" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F460" s="5" t="inlineStr">
@@ -19647,7 +19647,7 @@
       </c>
       <c r="E461" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F461" s="3" t="inlineStr">
@@ -20690,7 +20690,7 @@
       </c>
       <c r="E491" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F491" s="3" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="E492" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F492" s="5" t="inlineStr">
@@ -20764,7 +20764,7 @@
       </c>
       <c r="E493" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F493" s="3" t="inlineStr">
@@ -20838,7 +20838,7 @@
       </c>
       <c r="E495" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F495" s="3" t="inlineStr">
@@ -20875,7 +20875,7 @@
       </c>
       <c r="E496" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F496" s="5" t="inlineStr">
@@ -20949,7 +20949,7 @@
       </c>
       <c r="E498" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F498" s="5" t="inlineStr">
@@ -20986,7 +20986,7 @@
       </c>
       <c r="E499" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>14.00</t>
         </is>
       </c>
       <c r="F499" s="3" t="inlineStr">
@@ -21023,7 +21023,7 @@
       </c>
       <c r="E500" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>14.00</t>
         </is>
       </c>
       <c r="F500" s="5" t="inlineStr">
@@ -22103,7 +22103,7 @@
       </c>
       <c r="E531" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F531" s="3" t="inlineStr">
@@ -22140,7 +22140,7 @@
       </c>
       <c r="E532" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F532" s="5" t="inlineStr">
@@ -22177,7 +22177,7 @@
       </c>
       <c r="E533" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.50</t>
         </is>
       </c>
       <c r="F533" s="3" t="inlineStr">
@@ -22214,7 +22214,7 @@
       </c>
       <c r="E534" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F534" s="5" t="inlineStr">
@@ -22251,7 +22251,7 @@
       </c>
       <c r="E535" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F535" s="3" t="inlineStr">
@@ -22288,7 +22288,7 @@
       </c>
       <c r="E536" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="F536" s="5" t="inlineStr">
@@ -22325,7 +22325,7 @@
       </c>
       <c r="E537" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>23.00</t>
         </is>
       </c>
       <c r="F537" s="3" t="inlineStr">
@@ -22362,7 +22362,7 @@
       </c>
       <c r="E538" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>23.00</t>
         </is>
       </c>
       <c r="F538" s="5" t="inlineStr">
@@ -23479,7 +23479,7 @@
       </c>
       <c r="E570" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.50</t>
         </is>
       </c>
       <c r="F570" s="5" t="inlineStr">
@@ -23516,7 +23516,7 @@
       </c>
       <c r="E571" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F571" s="3" t="inlineStr">
@@ -23553,7 +23553,7 @@
       </c>
       <c r="E572" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.50</t>
         </is>
       </c>
       <c r="F572" s="5" t="inlineStr">
@@ -23590,7 +23590,7 @@
       </c>
       <c r="E573" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F573" s="3" t="inlineStr">
@@ -23627,7 +23627,7 @@
       </c>
       <c r="E574" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F574" s="5" t="inlineStr">
@@ -23664,7 +23664,7 @@
       </c>
       <c r="E575" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F575" s="3" t="inlineStr">
@@ -23701,7 +23701,7 @@
       </c>
       <c r="E576" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16.00</t>
         </is>
       </c>
       <c r="F576" s="5" t="inlineStr">
@@ -23738,7 +23738,7 @@
       </c>
       <c r="E577" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="F577" s="3" t="inlineStr">
@@ -23967,7 +23967,7 @@
       </c>
       <c r="E585" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="F585" s="3" t="inlineStr">
@@ -24670,7 +24670,7 @@
       </c>
       <c r="E604" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="F604" s="5" t="inlineStr">
@@ -24707,7 +24707,7 @@
       </c>
       <c r="E605" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.50</t>
         </is>
       </c>
       <c r="F605" s="3" t="inlineStr">
@@ -24781,7 +24781,7 @@
       </c>
       <c r="E607" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F607" s="3" t="inlineStr">
@@ -24818,7 +24818,7 @@
       </c>
       <c r="E608" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F608" s="5" t="inlineStr">
@@ -24855,7 +24855,7 @@
       </c>
       <c r="E609" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F609" s="3" t="inlineStr">
@@ -24892,7 +24892,7 @@
       </c>
       <c r="E610" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F610" s="5" t="inlineStr">
@@ -24929,7 +24929,7 @@
       </c>
       <c r="E611" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F611" s="3" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="E612" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="F612" s="5" t="inlineStr">
@@ -25003,7 +25003,7 @@
       </c>
       <c r="E613" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F613" s="3" t="inlineStr">
@@ -25972,7 +25972,7 @@
       </c>
       <c r="E641" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F641" s="3" t="inlineStr">
@@ -26009,7 +26009,7 @@
       </c>
       <c r="E642" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F642" s="5" t="inlineStr">
@@ -26046,7 +26046,7 @@
       </c>
       <c r="E643" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F643" s="3" t="inlineStr">
@@ -26120,7 +26120,7 @@
       </c>
       <c r="E645" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F645" s="3" t="inlineStr">
@@ -26194,7 +26194,7 @@
       </c>
       <c r="E647" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.00</t>
         </is>
       </c>
       <c r="F647" s="3" t="inlineStr">
@@ -26231,7 +26231,7 @@
       </c>
       <c r="E648" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F648" s="5" t="inlineStr">
@@ -26268,7 +26268,7 @@
       </c>
       <c r="E649" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F649" s="3" t="inlineStr">
@@ -26305,7 +26305,7 @@
       </c>
       <c r="E650" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>26.00</t>
         </is>
       </c>
       <c r="F650" s="5" t="inlineStr">
@@ -26423,7 +26423,7 @@
       </c>
       <c r="E655" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="F655" s="3" t="inlineStr">
@@ -27311,7 +27311,7 @@
       </c>
       <c r="E679" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F679" s="3" t="inlineStr">
@@ -27348,7 +27348,7 @@
       </c>
       <c r="E680" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.50</t>
         </is>
       </c>
       <c r="F680" s="5" t="inlineStr">
@@ -27385,7 +27385,7 @@
       </c>
       <c r="E681" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.50</t>
         </is>
       </c>
       <c r="F681" s="3" t="inlineStr">
@@ -27422,7 +27422,7 @@
       </c>
       <c r="E682" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.50</t>
         </is>
       </c>
       <c r="F682" s="5" t="inlineStr">
@@ -27496,7 +27496,7 @@
       </c>
       <c r="E684" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F684" s="5" t="inlineStr">
@@ -27533,7 +27533,7 @@
       </c>
       <c r="E685" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="F685" s="3" t="inlineStr">
@@ -27570,7 +27570,7 @@
       </c>
       <c r="E686" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F686" s="5" t="inlineStr">
@@ -27607,7 +27607,7 @@
       </c>
       <c r="E687" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19.00</t>
         </is>
       </c>
       <c r="F687" s="3" t="inlineStr">
@@ -27644,7 +27644,7 @@
       </c>
       <c r="E688" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="F688" s="5" t="inlineStr">
@@ -28687,7 +28687,7 @@
       </c>
       <c r="E718" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F718" s="5" t="inlineStr">
@@ -28761,7 +28761,7 @@
       </c>
       <c r="E720" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F720" s="5" t="inlineStr">
@@ -28798,7 +28798,7 @@
       </c>
       <c r="E721" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F721" s="3" t="inlineStr">
@@ -28835,7 +28835,7 @@
       </c>
       <c r="E722" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F722" s="5" t="inlineStr">
@@ -28872,7 +28872,7 @@
       </c>
       <c r="E723" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>14.00</t>
         </is>
       </c>
       <c r="F723" s="3" t="inlineStr">
@@ -28909,7 +28909,7 @@
       </c>
       <c r="E724" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="F724" s="5" t="inlineStr">
@@ -28946,7 +28946,7 @@
       </c>
       <c r="E725" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>22.00</t>
         </is>
       </c>
       <c r="F725" s="3" t="inlineStr">
@@ -28983,7 +28983,7 @@
       </c>
       <c r="E726" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F726" s="5" t="inlineStr">
@@ -29005,37 +29005,37 @@
       </c>
     </row>
     <row r="729" ht="15" customHeight="1">
-      <c r="A729" s="17" t="inlineStr">
+      <c r="A729" s="22" t="inlineStr">
         <is>
           <t>Portugal vs DR Congo</t>
         </is>
       </c>
-      <c r="B729" s="17" t="inlineStr">
-        <is>
-          <t>Double Chance 1X</t>
-        </is>
-      </c>
-      <c r="C729" s="3" t="inlineStr">
+      <c r="B729" s="22" t="inlineStr">
+        <is>
+          <t>Double Chance 1X *** ACCUMULATOR</t>
+        </is>
+      </c>
+      <c r="C729" s="23" t="inlineStr">
         <is>
           <t>1X</t>
         </is>
       </c>
-      <c r="D729" s="4" t="inlineStr">
+      <c r="D729" s="23" t="inlineStr">
         <is>
           <t>92.4%</t>
         </is>
       </c>
-      <c r="E729" s="3" t="inlineStr">
+      <c r="E729" s="23" t="inlineStr">
         <is>
           <t>1.08</t>
         </is>
       </c>
-      <c r="F729" s="3" t="inlineStr">
+      <c r="F729" s="23" t="inlineStr">
         <is>
           <t>dc</t>
         </is>
       </c>
-      <c r="G729" s="3" t="inlineStr">
+      <c r="G729" s="23" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
@@ -29079,37 +29079,37 @@
       </c>
     </row>
     <row r="731" ht="15" customHeight="1">
-      <c r="A731" s="22" t="inlineStr">
+      <c r="A731" s="17" t="inlineStr">
         <is>
           <t>Portugal vs DR Congo</t>
         </is>
       </c>
-      <c r="B731" s="22" t="inlineStr">
-        <is>
-          <t>Draw No Bet Portugal *** ACCUMULATOR</t>
-        </is>
-      </c>
-      <c r="C731" s="23" t="inlineStr">
+      <c r="B731" s="17" t="inlineStr">
+        <is>
+          <t>Draw No Bet Portugal</t>
+        </is>
+      </c>
+      <c r="C731" s="3" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="D731" s="23" t="inlineStr">
+      <c r="D731" s="4" t="inlineStr">
         <is>
           <t>90.0%</t>
         </is>
       </c>
-      <c r="E731" s="23" t="inlineStr">
-        <is>
-          <t>1.22</t>
-        </is>
-      </c>
-      <c r="F731" s="23" t="inlineStr">
+      <c r="E731" s="3" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="F731" s="3" t="inlineStr">
         <is>
           <t>dnb</t>
         </is>
       </c>
-      <c r="G731" s="23" t="inlineStr">
+      <c r="G731" s="3" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
@@ -29915,7 +29915,7 @@
       </c>
       <c r="E753" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F753" s="3" t="inlineStr">
@@ -29952,7 +29952,7 @@
       </c>
       <c r="E754" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="F754" s="5" t="inlineStr">
@@ -29989,7 +29989,7 @@
       </c>
       <c r="E755" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="F755" s="3" t="inlineStr">
@@ -30026,7 +30026,7 @@
       </c>
       <c r="E756" s="5" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F756" s="5" t="inlineStr">
@@ -30063,7 +30063,7 @@
       </c>
       <c r="E757" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F757" s="3" t="inlineStr">
@@ -30100,7 +30100,7 @@
       </c>
       <c r="E758" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.00</t>
         </is>
       </c>
       <c r="F758" s="5" t="inlineStr">
@@ -30137,7 +30137,7 @@
       </c>
       <c r="E759" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F759" s="3" t="inlineStr">
@@ -30211,7 +30211,7 @@
       </c>
       <c r="E761" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F761" s="3" t="inlineStr">
@@ -30248,7 +30248,7 @@
       </c>
       <c r="E762" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="F762" s="5" t="inlineStr">
@@ -30381,37 +30381,37 @@
       </c>
     </row>
     <row r="768" ht="15" customHeight="1">
-      <c r="A768" s="22" t="inlineStr">
+      <c r="A768" s="18" t="inlineStr">
         <is>
           <t>England vs Croatia</t>
         </is>
       </c>
-      <c r="B768" s="22" t="inlineStr">
-        <is>
-          <t>Draw No Bet England *** ACCUMULATOR</t>
-        </is>
-      </c>
-      <c r="C768" s="23" t="inlineStr">
+      <c r="B768" s="18" t="inlineStr">
+        <is>
+          <t>Draw No Bet England</t>
+        </is>
+      </c>
+      <c r="C768" s="5" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="D768" s="23" t="inlineStr">
+      <c r="D768" s="4" t="inlineStr">
         <is>
           <t>82.3%</t>
         </is>
       </c>
-      <c r="E768" s="23" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="F768" s="23" t="inlineStr">
+      <c r="E768" s="5" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="F768" s="5" t="inlineStr">
         <is>
           <t>dnb</t>
         </is>
       </c>
-      <c r="G768" s="23" t="inlineStr">
+      <c r="G768" s="5" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
@@ -30751,37 +30751,37 @@
       </c>
     </row>
     <row r="778" ht="15" customHeight="1">
-      <c r="A778" s="18" t="inlineStr">
+      <c r="A778" s="22" t="inlineStr">
         <is>
           <t>England vs Croatia</t>
         </is>
       </c>
-      <c r="B778" s="18" t="inlineStr">
-        <is>
-          <t>1X2 Result</t>
-        </is>
-      </c>
-      <c r="C778" s="5" t="inlineStr">
+      <c r="B778" s="22" t="inlineStr">
+        <is>
+          <t>1X2 Result *** ACCUMULATOR</t>
+        </is>
+      </c>
+      <c r="C778" s="23" t="inlineStr">
         <is>
           <t>1 (England)</t>
         </is>
       </c>
-      <c r="D778" s="15" t="inlineStr">
+      <c r="D778" s="23" t="inlineStr">
         <is>
           <t>62.8%</t>
         </is>
       </c>
-      <c r="E778" s="5" t="inlineStr">
+      <c r="E778" s="23" t="inlineStr">
         <is>
           <t>1.72</t>
         </is>
       </c>
-      <c r="F778" s="5" t="inlineStr">
+      <c r="F778" s="23" t="inlineStr">
         <is>
           <t>result</t>
         </is>
       </c>
-      <c r="G778" s="5" t="inlineStr">
+      <c r="G778" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -31180,7 +31180,7 @@
       </c>
       <c r="E789" s="3" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="F789" s="3" t="inlineStr">
@@ -31254,7 +31254,7 @@
       </c>
       <c r="E791" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F791" s="3" t="inlineStr">
@@ -31291,7 +31291,7 @@
       </c>
       <c r="E792" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="F792" s="5" t="inlineStr">
@@ -31328,7 +31328,7 @@
       </c>
       <c r="E793" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F793" s="3" t="inlineStr">
@@ -31365,7 +31365,7 @@
       </c>
       <c r="E794" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F794" s="5" t="inlineStr">
@@ -31402,7 +31402,7 @@
       </c>
       <c r="E795" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F795" s="3" t="inlineStr">
@@ -31439,7 +31439,7 @@
       </c>
       <c r="E796" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F796" s="5" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="E797" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="F797" s="3" t="inlineStr">
@@ -31513,7 +31513,7 @@
       </c>
       <c r="E798" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="F798" s="5" t="inlineStr">
@@ -32482,7 +32482,7 @@
       </c>
       <c r="E826" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F826" s="5" t="inlineStr">
@@ -32519,7 +32519,7 @@
       </c>
       <c r="E827" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F827" s="3" t="inlineStr">
@@ -32556,7 +32556,7 @@
       </c>
       <c r="E828" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="F828" s="5" t="inlineStr">
@@ -32593,7 +32593,7 @@
       </c>
       <c r="E829" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="F829" s="3" t="inlineStr">
@@ -32630,7 +32630,7 @@
       </c>
       <c r="E830" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="F830" s="5" t="inlineStr">
@@ -32667,7 +32667,7 @@
       </c>
       <c r="E831" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F831" s="3" t="inlineStr">
@@ -32704,7 +32704,7 @@
       </c>
       <c r="E832" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16.00</t>
         </is>
       </c>
       <c r="F832" s="5" t="inlineStr">
@@ -32741,7 +32741,7 @@
       </c>
       <c r="E833" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F833" s="3" t="inlineStr">
@@ -33747,7 +33747,7 @@
       </c>
       <c r="E862" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F862" s="5" t="inlineStr">
@@ -33784,7 +33784,7 @@
       </c>
       <c r="E863" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="F863" s="3" t="inlineStr">
@@ -33858,7 +33858,7 @@
       </c>
       <c r="E865" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="F865" s="3" t="inlineStr">
@@ -33895,7 +33895,7 @@
       </c>
       <c r="E866" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.50</t>
         </is>
       </c>
       <c r="F866" s="5" t="inlineStr">
@@ -33932,7 +33932,7 @@
       </c>
       <c r="E867" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="F867" s="3" t="inlineStr">
@@ -33969,7 +33969,7 @@
       </c>
       <c r="E868" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18.00</t>
         </is>
       </c>
       <c r="F868" s="5" t="inlineStr">
@@ -34006,7 +34006,7 @@
       </c>
       <c r="E869" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>28.00</t>
         </is>
       </c>
       <c r="F869" s="3" t="inlineStr">
@@ -34043,7 +34043,7 @@
       </c>
       <c r="E870" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F870" s="5" t="inlineStr">
@@ -35168,22 +35168,22 @@
       </c>
       <c r="D39" s="25" t="inlineStr">
         <is>
-          <t>Double Chance X2</t>
+          <t>Draw No Bet Japan</t>
         </is>
       </c>
       <c r="E39" s="24" t="inlineStr">
         <is>
-          <t>X2</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>74.1%</t>
+          <t>57.3%</t>
         </is>
       </c>
       <c r="G39" s="24" t="inlineStr">
         <is>
-          <t>dc</t>
+          <t>dnb</t>
         </is>
       </c>
     </row>
@@ -36389,22 +36389,22 @@
       </c>
       <c r="D83" s="25" t="inlineStr">
         <is>
-          <t>Draw No Bet Portugal</t>
+          <t>Double Chance 1X</t>
         </is>
       </c>
       <c r="E83" s="24" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>1X</t>
         </is>
       </c>
       <c r="F83" s="24" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>92.4%</t>
         </is>
       </c>
       <c r="G83" s="24" t="inlineStr">
         <is>
-          <t>dnb</t>
+          <t>dc</t>
         </is>
       </c>
     </row>
@@ -36500,22 +36500,22 @@
       </c>
       <c r="D87" s="25" t="inlineStr">
         <is>
-          <t>Draw No Bet England</t>
+          <t>1X2 Result</t>
         </is>
       </c>
       <c r="E87" s="24" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>1 (England)</t>
         </is>
       </c>
       <c r="F87" s="24" t="inlineStr">
         <is>
-          <t>82.3%</t>
+          <t>62.8%</t>
         </is>
       </c>
       <c r="G87" s="24" t="inlineStr">
         <is>
-          <t>dnb</t>
+          <t>result</t>
         </is>
       </c>
     </row>
@@ -37125,22 +37125,22 @@
       </c>
       <c r="D9" s="30" t="inlineStr">
         <is>
-          <t>GG (Both Teams Score)</t>
+          <t>Correct Score 2-1</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Da</t>
-        </is>
-      </c>
-      <c r="F9" s="28" t="inlineStr">
-        <is>
-          <t>52.7%</t>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>gg</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37162,22 +37162,22 @@
       </c>
       <c r="D10" s="31" t="inlineStr">
         <is>
-          <t>1X2 Result</t>
+          <t>Correct Score 2-1</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>2 (Turkey)</t>
-        </is>
-      </c>
-      <c r="F10" s="26" t="inlineStr">
-        <is>
-          <t>64.0%</t>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>7.3%</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37199,22 +37199,22 @@
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
-          <t>Goals O/U 2.5</t>
+          <t>Correct Score 1-1</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Under 2.5</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="inlineStr">
-        <is>
-          <t>50.6%</t>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>goals_ou</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37236,22 +37236,22 @@
       </c>
       <c r="D12" s="31" t="inlineStr">
         <is>
-          <t>1X2 Result</t>
+          <t>Draw No Bet Japan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>X (egal)</t>
-        </is>
-      </c>
-      <c r="F12" s="32" t="inlineStr">
-        <is>
-          <t>39.2%</t>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>57.3%</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>dnb</t>
         </is>
       </c>
     </row>
@@ -37310,22 +37310,22 @@
       </c>
       <c r="D14" s="31" t="inlineStr">
         <is>
-          <t>1X2 Result</t>
+          <t>Correct Score 0-2</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>1 (Sweden)</t>
-        </is>
-      </c>
-      <c r="F14" s="26" t="inlineStr">
-        <is>
-          <t>61.6%</t>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37347,22 +37347,22 @@
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>Goals O/U 3.5</t>
+          <t>Correct Score 1-1</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Under 3.5</t>
-        </is>
-      </c>
-      <c r="F15" s="26" t="inlineStr">
-        <is>
-          <t>72.8%</t>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>goals_ou</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37421,22 +37421,22 @@
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>Double Chance 1X</t>
+          <t>Correct Score 2-1</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>1X</t>
-        </is>
-      </c>
-      <c r="F17" s="28" t="inlineStr">
-        <is>
-          <t>46.8%</t>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>dc</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37569,22 +37569,22 @@
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>Goals O/U 2.5</t>
+          <t>Correct Score 0-1</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Under 2.5</t>
-        </is>
-      </c>
-      <c r="F21" s="28" t="inlineStr">
-        <is>
-          <t>55.2%</t>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>goals_ou</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37606,22 +37606,22 @@
       </c>
       <c r="D22" s="31" t="inlineStr">
         <is>
-          <t>Draw No Bet Jordan</t>
+          <t>Correct Score 0-1</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Win</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="F22" s="32" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>dnb</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37643,22 +37643,22 @@
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>Draw No Bet Portugal</t>
+          <t>Correct Score 1-1</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="F23" s="24" t="inlineStr">
-        <is>
-          <t>90.0%</t>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>dnb</t>
+          <t>correct</t>
         </is>
       </c>
     </row>
@@ -37680,22 +37680,22 @@
       </c>
       <c r="D24" s="31" t="inlineStr">
         <is>
-          <t>Draw No Bet England</t>
+          <t>Correct Score 1-2</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="F24" s="24" t="inlineStr">
-        <is>
-          <t>82.3%</t>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>dnb</t>
+          <t>correct</t>
         </is>
       </c>
     </row>

</xml_diff>